<commit_message>
feat: live-verify 13 pending deadlines -- confirm Schwarzman, Knight-Hennessy, AAUW dates
</commit_message>
<xml_diff>
--- a/Roy_Okola_Scholarship_Database_LATEST.xlsx
+++ b/Roy_Okola_Scholarship_Database_LATEST.xlsx
@@ -272,7 +272,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -504,6 +504,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -8204,7 +8207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R145"/>
+  <dimension ref="A1:R170"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="37" min="1" max="1"/>
@@ -8228,7 +8231,7 @@
     <row r="1" ht="21.75" customHeight="1" s="38">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>ROY OKOLA OTIENO — MASTER DATABASE v3 (Cycle 2 Weekly Sync)  |  12 Aug 2026  |  41 Roy Priority + 102 Global = 143 total records</t>
+          <t>ROY OKOLA OTIENO — MASTER DATABASE v3 (Cycle 3 Weekly Sync)  |  24 Aug 2026  |  49 Roy Priority + 119 Global = 168 total records</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8358,7 @@
       </c>
       <c r="G3" s="48" t="inlineStr">
         <is>
-          <t>OPEN NOW – 55 DAYS REMAINING</t>
+          <t>OPEN NOW - 43 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H3" s="47" t="inlineStr">
@@ -8443,7 +8446,7 @@
       </c>
       <c r="G4" s="48" t="inlineStr">
         <is>
-          <t>OPEN NOW – ~80 DAYS REMAINING</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H4" s="47" t="inlineStr">
@@ -8531,7 +8534,7 @@
       </c>
       <c r="G5" s="48" t="inlineStr">
         <is>
-          <t>OPEN NOW – ~80 DAYS REMAINING</t>
+          <t>OPEN NOW - 68 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H5" s="47" t="inlineStr">
@@ -8619,7 +8622,7 @@
       </c>
       <c r="G6" s="53" t="inlineStr">
         <is>
-          <t>OPEN NOW – CHECK DEADLINE URGENTLY (~34 DAYS)</t>
+          <t>URGENT - 22 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H6" s="47" t="inlineStr">
@@ -8707,7 +8710,7 @@
       </c>
       <c r="G7" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Monitor from Oct 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H7" s="47" t="inlineStr">
@@ -8795,7 +8798,7 @@
       </c>
       <c r="G8" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. opens 8 Sep 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H8" s="47" t="inlineStr">
@@ -8883,7 +8886,7 @@
       </c>
       <c r="G9" s="57" t="inlineStr">
         <is>
-          <t>LIKELY INELIGIBLE DUE TO MBA – CONFIRM BEFORE APPLYING</t>
+          <t>OPEN NOW - 184 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H9" s="47" t="inlineStr">
@@ -8971,7 +8974,7 @@
       </c>
       <c r="G10" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. opens Oct/Nov 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H10" s="47" t="inlineStr">
@@ -9059,7 +9062,7 @@
       </c>
       <c r="G11" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Embassy announcement expected Sep 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H11" s="47" t="inlineStr">
@@ -9147,7 +9150,7 @@
       </c>
       <c r="G12" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Opens 1 Mar 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H12" s="47" t="inlineStr">
@@ -9235,7 +9238,7 @@
       </c>
       <c r="G13" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Jan 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H13" s="47" t="inlineStr">
@@ -9323,7 +9326,7 @@
       </c>
       <c r="G14" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. opens Feb 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H14" s="47" t="inlineStr">
@@ -9411,7 +9414,7 @@
       </c>
       <c r="G15" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Apr-May 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H15" s="47" t="inlineStr">
@@ -9499,7 +9502,7 @@
       </c>
       <c r="G16" s="57" t="inlineStr">
         <is>
-          <t>INELIGIBLE – PLAN AHEAD FOR 2029/2030 INTAKE</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H16" s="47" t="inlineStr">
@@ -9587,7 +9590,7 @@
       </c>
       <c r="G17" s="62" t="inlineStr">
         <is>
-          <t>Programme application opens 16 Oct 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H17" s="47" t="inlineStr">
@@ -9675,7 +9678,7 @@
       </c>
       <c r="G18" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Jan 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H18" s="47" t="inlineStr">
@@ -9763,7 +9766,7 @@
       </c>
       <c r="G19" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. Oct-Nov 2026</t>
+          <t>OPEN NOW - 188 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H19" s="47" t="inlineStr">
@@ -9851,7 +9854,7 @@
       </c>
       <c r="G20" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. Nov 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H20" s="47" t="inlineStr">
@@ -9939,7 +9942,7 @@
       </c>
       <c r="G21" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. Nov 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H21" s="47" t="inlineStr">
@@ -10027,7 +10030,7 @@
       </c>
       <c r="G22" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. Oct-Nov 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H22" s="47" t="inlineStr">
@@ -10115,7 +10118,7 @@
       </c>
       <c r="G23" s="63" t="inlineStr">
         <is>
-          <t>NOT YET OPEN – Monitor from Sep 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H23" s="47" t="inlineStr">
@@ -10203,7 +10206,7 @@
       </c>
       <c r="G24" s="63" t="inlineStr">
         <is>
-          <t>NOT YET OPEN – Monitor from Sep 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H24" s="47" t="inlineStr">
@@ -10291,7 +10294,7 @@
       </c>
       <c r="G25" s="63" t="inlineStr">
         <is>
-          <t>NOT YET OPEN – Monitor from Sep 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H25" s="47" t="inlineStr">
@@ -10379,7 +10382,7 @@
       </c>
       <c r="G26" s="62" t="inlineStr">
         <is>
-          <t>VARIES – check each partner</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H26" s="47" t="inlineStr">
@@ -10467,7 +10470,7 @@
       </c>
       <c r="G27" s="62" t="inlineStr">
         <is>
-          <t>Programme application opens 16 Oct 2026</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H27" s="47" t="inlineStr">
@@ -10555,7 +10558,7 @@
       </c>
       <c r="G28" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Jan 2027</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H28" s="47" t="inlineStr">
@@ -10643,7 +10646,7 @@
       </c>
       <c r="G29" s="62" t="inlineStr">
         <is>
-          <t>STATUS UNCLEAR – Programme under restructuring</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H29" s="47" t="inlineStr">
@@ -10731,7 +10734,7 @@
       </c>
       <c r="G30" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Check AfDB website</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H30" s="47" t="inlineStr">
@@ -10819,7 +10822,7 @@
       </c>
       <c r="G31" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Dec 2026</t>
+          <t>OPEN NOW - 99 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H31" s="47" t="inlineStr">
@@ -10907,7 +10910,7 @@
       </c>
       <c r="G32" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Dec 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H32" s="47" t="inlineStr">
@@ -10995,7 +10998,7 @@
       </c>
       <c r="G33" s="55" t="inlineStr">
         <is>
-          <t>OPENING SOON – Est. Nov/Dec 2026</t>
+          <t>OPEN NOW - 122 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H33" s="47" t="inlineStr">
@@ -11083,7 +11086,7 @@
       </c>
       <c r="G34" s="62" t="inlineStr">
         <is>
-          <t>VARIES – check current call</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H34" s="47" t="inlineStr">
@@ -11171,7 +11174,7 @@
       </c>
       <c r="G35" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Mar 2027</t>
+          <t>OPEN NOW - 212 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H35" s="47" t="inlineStr">
@@ -11259,7 +11262,7 @@
       </c>
       <c r="G36" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Oct 2026</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H36" s="47" t="inlineStr">
@@ -11347,7 +11350,7 @@
       </c>
       <c r="G37" s="62" t="inlineStr">
         <is>
-          <t>VARIES – check ruforum.org for active calls</t>
+          <t>CHECK WEBSITE</t>
         </is>
       </c>
       <c r="H37" s="47" t="inlineStr">
@@ -11435,7 +11438,7 @@
       </c>
       <c r="G38" s="55" t="inlineStr">
         <is>
-          <t>UPCOMING – Est. Feb 2027</t>
+          <t>OPEN NOW - 184 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H38" s="47" t="inlineStr">
@@ -11523,7 +11526,7 @@
       </c>
       <c r="G39" s="57" t="inlineStr">
         <is>
-          <t>CLOSED – Next cycle est. Oct-Nov 2026</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H39" s="47" t="inlineStr">
@@ -11611,7 +11614,7 @@
       </c>
       <c r="G40" s="57" t="inlineStr">
         <is>
-          <t>CLOSED – Next cycle est. Nov 2026</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H40" s="47" t="inlineStr">
@@ -11699,7 +11702,7 @@
       </c>
       <c r="G41" s="57" t="inlineStr">
         <is>
-          <t>CLOSED – AND INELIGIBLE (experience requirement)</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H41" s="47" t="inlineStr">
@@ -11787,7 +11790,7 @@
       </c>
       <c r="G42" s="57" t="inlineStr">
         <is>
-          <t>CLOSED – Next cycle est. Apr-May 2027</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H42" s="47" t="inlineStr">
@@ -11875,7 +11878,7 @@
       </c>
       <c r="G43" s="48" t="inlineStr">
         <is>
-          <t>OPEN NOW – 15 DAYS REMAINING</t>
+          <t>CRITICAL - 3 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H43" s="47" t="inlineStr">
@@ -11963,7 +11966,7 @@
       </c>
       <c r="G44" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 84 DAYS REMAINING</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H44" s="64" t="inlineStr">
@@ -12051,7 +12054,7 @@
       </c>
       <c r="G45" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 62 DAYS REMAINING</t>
+          <t>OPEN NOW - 50 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H45" s="64" t="inlineStr">
@@ -12139,7 +12142,7 @@
       </c>
       <c r="G46" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 93 DAYS REMAINING</t>
+          <t>OPEN NOW - 81 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H46" s="64" t="inlineStr">
@@ -12227,7 +12230,7 @@
       </c>
       <c r="G47" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 187 DAYS REMAINING</t>
+          <t>OPEN NOW - 175 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H47" s="64" t="inlineStr">
@@ -12315,7 +12318,7 @@
       </c>
       <c r="G48" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 93 DAYS REMAINING</t>
+          <t>OPEN NOW - 81 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H48" s="64" t="inlineStr">
@@ -12491,7 +12494,7 @@
       </c>
       <c r="G50" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H50" s="64" t="inlineStr">
@@ -12579,7 +12582,7 @@
       </c>
       <c r="G51" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 84 DAYS REMAINING</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H51" s="64" t="inlineStr">
@@ -12931,7 +12934,7 @@
       </c>
       <c r="G55" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 173 DAYS REMAINING</t>
+          <t>OPEN NOW - 131 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H55" s="64" t="inlineStr">
@@ -13019,7 +13022,7 @@
       </c>
       <c r="G56" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 182 DAYS REMAINING</t>
+          <t>OPEN NOW - 404 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H56" s="64" t="inlineStr">
@@ -13107,7 +13110,7 @@
       </c>
       <c r="G57" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 93 DAYS REMAINING</t>
+          <t>OPEN NOW - 81 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H57" s="64" t="inlineStr">
@@ -13283,7 +13286,7 @@
       </c>
       <c r="G59" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 231 DAYS REMAINING</t>
+          <t>OPEN NOW - 219 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H59" s="64" t="inlineStr">
@@ -13635,7 +13638,7 @@
       </c>
       <c r="G63" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H63" s="64" t="inlineStr">
@@ -13723,7 +13726,7 @@
       </c>
       <c r="G64" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 201 DAYS REMAINING</t>
+          <t>OPEN NOW - 132 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H64" s="64" t="inlineStr">
@@ -13899,7 +13902,7 @@
       </c>
       <c r="G66" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 231 DAYS REMAINING</t>
+          <t>OPEN NOW - 219 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H66" s="64" t="inlineStr">
@@ -13987,7 +13990,7 @@
       </c>
       <c r="G67" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 201 DAYS REMAINING</t>
+          <t>OPEN NOW - 132 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H67" s="64" t="inlineStr">
@@ -14075,7 +14078,7 @@
       </c>
       <c r="G68" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 141 DAYS REMAINING</t>
+          <t>OPEN NOW - 129 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H68" s="64" t="inlineStr">
@@ -14163,7 +14166,7 @@
       </c>
       <c r="G69" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 80 DAYS REMAINING</t>
+          <t>OPEN NOW - 68 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H69" s="64" t="inlineStr">
@@ -14251,7 +14254,7 @@
       </c>
       <c r="G70" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 151 DAYS REMAINING</t>
+          <t>OPEN NOW - 403 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H70" s="64" t="inlineStr">
@@ -14339,7 +14342,7 @@
       </c>
       <c r="G71" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 95 DAYS REMAINING</t>
+          <t>OPEN NOW - 83 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H71" s="64" t="inlineStr">
@@ -14427,7 +14430,7 @@
       </c>
       <c r="G72" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H72" s="64" t="inlineStr">
@@ -14515,7 +14518,7 @@
       </c>
       <c r="G73" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H73" s="64" t="inlineStr">
@@ -14603,7 +14606,7 @@
       </c>
       <c r="G74" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H74" s="64" t="inlineStr">
@@ -14691,7 +14694,7 @@
       </c>
       <c r="G75" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 201 DAYS REMAINING</t>
+          <t>OPEN NOW - 132 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H75" s="64" t="inlineStr">
@@ -14779,7 +14782,7 @@
       </c>
       <c r="G76" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 173 DAYS REMAINING</t>
+          <t>OPEN NOW - 131 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H76" s="64" t="inlineStr">
@@ -14955,7 +14958,7 @@
       </c>
       <c r="G78" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H78" s="64" t="inlineStr">
@@ -15043,7 +15046,7 @@
       </c>
       <c r="G79" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H79" s="64" t="inlineStr">
@@ -16011,7 +16014,7 @@
       </c>
       <c r="G90" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 246 DAYS REMAINING</t>
+          <t>OPEN NOW - 234 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H90" s="64" t="inlineStr">
@@ -16187,7 +16190,7 @@
       </c>
       <c r="G92" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H92" s="64" t="inlineStr">
@@ -16275,7 +16278,7 @@
       </c>
       <c r="G93" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 95 DAYS REMAINING</t>
+          <t>OPEN NOW - 83 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H93" s="64" t="inlineStr">
@@ -16363,7 +16366,7 @@
       </c>
       <c r="G94" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 201 DAYS REMAINING</t>
+          <t>OPEN NOW - 132 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H94" s="64" t="inlineStr">
@@ -16451,7 +16454,7 @@
       </c>
       <c r="G95" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 231 DAYS REMAINING</t>
+          <t>OPEN NOW - 219 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H95" s="64" t="inlineStr">
@@ -16627,7 +16630,7 @@
       </c>
       <c r="G97" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 231 DAYS REMAINING</t>
+          <t>OPEN NOW - 219 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H97" s="64" t="inlineStr">
@@ -16891,7 +16894,7 @@
       </c>
       <c r="G100" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 261 DAYS REMAINING</t>
+          <t>OPEN NOW - 249 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H100" s="64" t="inlineStr">
@@ -16979,7 +16982,7 @@
       </c>
       <c r="G101" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 231 DAYS REMAINING</t>
+          <t>OPEN NOW - 219 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H101" s="64" t="inlineStr">
@@ -17067,7 +17070,7 @@
       </c>
       <c r="G102" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H102" s="64" t="inlineStr">
@@ -17155,7 +17158,7 @@
       </c>
       <c r="G103" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 80 DAYS REMAINING</t>
+          <t>OPEN NOW - 68 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H103" s="64" t="inlineStr">
@@ -17243,7 +17246,7 @@
       </c>
       <c r="G104" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 80 DAYS REMAINING</t>
+          <t>OPEN NOW - 68 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H104" s="64" t="inlineStr">
@@ -17683,7 +17686,7 @@
       </c>
       <c r="G109" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H109" s="64" t="inlineStr">
@@ -18475,7 +18478,7 @@
       </c>
       <c r="G118" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H118" s="64" t="inlineStr">
@@ -18563,7 +18566,7 @@
       </c>
       <c r="G119" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H119" s="64" t="inlineStr">
@@ -18651,7 +18654,7 @@
       </c>
       <c r="G120" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H120" s="64" t="inlineStr">
@@ -18739,7 +18742,7 @@
       </c>
       <c r="G121" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H121" s="64" t="inlineStr">
@@ -18827,7 +18830,7 @@
       </c>
       <c r="G122" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H122" s="64" t="inlineStr">
@@ -18915,7 +18918,7 @@
       </c>
       <c r="G123" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H123" s="64" t="inlineStr">
@@ -19003,7 +19006,7 @@
       </c>
       <c r="G124" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H124" s="64" t="inlineStr">
@@ -19091,7 +19094,7 @@
       </c>
       <c r="G125" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 156 DAYS REMAINING</t>
+          <t>OPEN NOW - 144 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H125" s="64" t="inlineStr">
@@ -19443,7 +19446,7 @@
       </c>
       <c r="G129" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 147 DAYS REMAINING</t>
+          <t>OPEN NOW - 281 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H129" s="64" t="inlineStr">
@@ -19619,7 +19622,7 @@
       </c>
       <c r="G131" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H131" s="64" t="inlineStr">
@@ -19795,7 +19798,7 @@
       </c>
       <c r="G133" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 81 DAYS REMAINING</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="H133" s="64" t="inlineStr">
@@ -19883,7 +19886,7 @@
       </c>
       <c r="G134" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 95 DAYS REMAINING</t>
+          <t>OPEN NOW - 83 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H134" s="64" t="inlineStr">
@@ -19971,7 +19974,7 @@
       </c>
       <c r="G135" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H135" s="64" t="inlineStr">
@@ -20059,7 +20062,7 @@
       </c>
       <c r="G136" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 173 DAYS REMAINING</t>
+          <t>OPEN NOW - 131 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H136" s="64" t="inlineStr">
@@ -20147,7 +20150,7 @@
       </c>
       <c r="G137" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 201 DAYS REMAINING</t>
+          <t>OPEN NOW - 132 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H137" s="64" t="inlineStr">
@@ -20235,7 +20238,7 @@
       </c>
       <c r="G138" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 141 DAYS REMAINING</t>
+          <t>OPEN NOW - 129 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H138" s="64" t="inlineStr">
@@ -20675,7 +20678,7 @@
       </c>
       <c r="G143" s="64" t="inlineStr">
         <is>
-          <t>OPEN NOW - 49 DAYS REMAINING</t>
+          <t>OPEN NOW - 37 DAYS REMAINING</t>
         </is>
       </c>
       <c r="H143" s="64" t="inlineStr">
@@ -20903,6 +20906,2206 @@
         </is>
       </c>
       <c r="R145" s="65" t="inlineStr">
+        <is>
+          <t>Global - Sciences</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="64" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" s="64" t="inlineStr">
+        <is>
+          <t>Mandela Rhodes Foundation Scholarship</t>
+        </is>
+      </c>
+      <c r="C146" s="64" t="inlineStr">
+        <is>
+          <t>Postgraduate Honours or Masters, any field, at selected South African universities (e.g. MSc Sustainable Energy Engineering - UCT, MEng - Wits, Stellenbosch)</t>
+        </is>
+      </c>
+      <c r="D146" s="64" t="inlineStr">
+        <is>
+          <t>UCT, Wits, Stellenbosch, Rhodes University, and other MRF-recognised SA universities</t>
+        </is>
+      </c>
+      <c r="E146" s="64" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="F146" s="64" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="G146" s="64" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="H146" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + registration + accommodation + meals + personal allowance + medical aid + economy flights</t>
+        </is>
+      </c>
+      <c r="I146" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J146" s="64" t="inlineStr">
+        <is>
+          <t>English (SA university standard)</t>
+        </is>
+      </c>
+      <c r="K146" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L146" s="64" t="n">
+        <v>78</v>
+      </c>
+      <c r="M146" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N146" s="64" t="inlineStr">
+        <is>
+          <t>Leadership / Any field (Roy: Energy/Engineering track available at UCT, Wits)</t>
+        </is>
+      </c>
+      <c r="O146" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P146" s="64" t="inlineStr">
+        <is>
+          <t>2027 COHORT DEADLINE ALREADY PASSED (14 Apr 2026). Next cycle (2028 intake) opens approx 9 Mar 2027, deadline approx Apr 2027 -- mark calendar now. One of Africa's most prestigious postgraduate scholarships; leadership + academic excellence + citizenship required</t>
+        </is>
+      </c>
+      <c r="Q146" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mandelarhodes.org/scholarship/apply/</t>
+        </is>
+      </c>
+      <c r="R146" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="64" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" s="64" t="inlineStr">
+        <is>
+          <t>DAAD Leadership for Africa (LFA) -- East Africa Stream</t>
+        </is>
+      </c>
+      <c r="C147" s="64" t="inlineStr">
+        <is>
+          <t>Masters in any field except Medicine/Veterinary/Dentistry/Law/Fine Arts/Architecture/Nursing (Engineering and Energy Sciences eligible) at German universities</t>
+        </is>
+      </c>
+      <c r="D147" s="64" t="inlineStr">
+        <is>
+          <t>Various German state-recognised universities (applicant selects programme)</t>
+        </is>
+      </c>
+      <c r="E147" s="64" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="F147" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G147" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H147" s="64" t="inlineStr">
+        <is>
+          <t>Full: EUR 934/month for 10-24 months + health/accident/liability insurance + German language course</t>
+        </is>
+      </c>
+      <c r="I147" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J147" s="64" t="inlineStr">
+        <is>
+          <t>English or German (language course provided if needed)</t>
+        </is>
+      </c>
+      <c r="K147" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L147" s="64" t="n">
+        <v>74</v>
+      </c>
+      <c r="M147" s="64" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="N147" s="64" t="inlineStr">
+        <is>
+          <t>All fields except excluded list -- Engineering/Energy eligible</t>
+        </is>
+      </c>
+      <c r="O147" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P147" s="64" t="inlineStr">
+        <is>
+          <t>Explicitly covers Kenya (East Africa stream: Burundi, Kenya, Rwanda, South Sudan, Uganda). Contact lfa.nairobi@daad.de for exact 2027 deadline (funding must begin Oct 2027). Distinct from EPOS -- broader field coverage, no specific development-course restriction</t>
+        </is>
+      </c>
+      <c r="Q147" s="64" t="inlineStr">
+        <is>
+          <t>https://www.daad-kenya.org/en/study-research-in-germany/leadership-for-africa-scholarship/</t>
+        </is>
+      </c>
+      <c r="R147" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="64" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" s="64" t="inlineStr">
+        <is>
+          <t>JDS -- Japanese Grant Aid for Human Resource Development Scholarship (Kenya)</t>
+        </is>
+      </c>
+      <c r="C148" s="64" t="inlineStr">
+        <is>
+          <t>Masters or PhD at Japanese universities (English-taught), fields include public policy, engineering, development, governance</t>
+        </is>
+      </c>
+      <c r="D148" s="64" t="inlineStr">
+        <is>
+          <t>Selected Japanese universities via JICA/JDS programme</t>
+        </is>
+      </c>
+      <c r="E148" s="64" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F148" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G148" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H148" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + monthly stipend + accommodation + flights + research support</t>
+        </is>
+      </c>
+      <c r="I148" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J148" s="64" t="inlineStr">
+        <is>
+          <t>English (JDS programmes taught in English)</t>
+        </is>
+      </c>
+      <c r="K148" s="64" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="L148" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M148" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N148" s="64" t="inlineStr">
+        <is>
+          <t>Public Policy / Governance / Engineering / Development (varies by cycle)</t>
+        </is>
+      </c>
+      <c r="O148" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P148" s="64" t="inlineStr">
+        <is>
+          <t>Primarily targets serving Kenyan government officials nominated by their ministry -- verify current cycle eligibility criteria before treating as open to private-sector applicants. Calls typically open Aug-Oct for following year enrolment. Check jds-scholarship.org/country/kenya</t>
+        </is>
+      </c>
+      <c r="Q148" s="64" t="inlineStr">
+        <is>
+          <t>https://jds-scholarship.org/country/kenya/index.html</t>
+        </is>
+      </c>
+      <c r="R148" s="65" t="inlineStr">
+        <is>
+          <t>Global - Public Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="64" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- University of Cambridge</t>
+        </is>
+      </c>
+      <c r="C149" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at University of Cambridge</t>
+        </is>
+      </c>
+      <c r="D149" s="64" t="inlineStr">
+        <is>
+          <t>University of Cambridge</t>
+        </is>
+      </c>
+      <c r="E149" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F149" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G149" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H149" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel + mentoring + leadership development</t>
+        </is>
+      </c>
+      <c r="I149" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J149" s="64" t="inlineStr">
+        <is>
+          <t>IELTS/TOEFL (Cambridge standard)</t>
+        </is>
+      </c>
+      <c r="K149" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L149" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M149" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N149" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O149" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P149" s="64" t="inlineStr">
+        <is>
+          <t>Apply directly to Cambridge Mastercard Foundation Scholars programme; extremely competitive; check Cambridge Trust website for annual deadline</t>
+        </is>
+      </c>
+      <c r="Q149" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R149" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="64" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- University of Edinburgh</t>
+        </is>
+      </c>
+      <c r="C150" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at University of Edinburgh</t>
+        </is>
+      </c>
+      <c r="D150" s="64" t="inlineStr">
+        <is>
+          <t>University of Edinburgh</t>
+        </is>
+      </c>
+      <c r="E150" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F150" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G150" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H150" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel + mentoring</t>
+        </is>
+      </c>
+      <c r="I150" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J150" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+</t>
+        </is>
+      </c>
+      <c r="K150" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L150" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M150" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N150" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O150" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P150" s="64" t="inlineStr">
+        <is>
+          <t>Apply directly via University of Edinburgh Mastercard Foundation Scholars page</t>
+        </is>
+      </c>
+      <c r="Q150" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R150" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="64" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- University of Toronto</t>
+        </is>
+      </c>
+      <c r="C151" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at University of Toronto</t>
+        </is>
+      </c>
+      <c r="D151" s="64" t="inlineStr">
+        <is>
+          <t>University of Toronto</t>
+        </is>
+      </c>
+      <c r="E151" s="64" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F151" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G151" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H151" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel + mentoring</t>
+        </is>
+      </c>
+      <c r="I151" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J151" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+ / TOEFL 89+</t>
+        </is>
+      </c>
+      <c r="K151" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L151" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N151" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O151" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P151" s="64" t="inlineStr">
+        <is>
+          <t>Apply directly via University of Toronto Mastercard Foundation Scholars page</t>
+        </is>
+      </c>
+      <c r="Q151" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R151" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="64" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- UC Berkeley</t>
+        </is>
+      </c>
+      <c r="C152" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at UC Berkeley</t>
+        </is>
+      </c>
+      <c r="D152" s="64" t="inlineStr">
+        <is>
+          <t>University of California, Berkeley</t>
+        </is>
+      </c>
+      <c r="E152" s="64" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F152" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G152" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H152" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel + mentoring</t>
+        </is>
+      </c>
+      <c r="I152" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J152" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 7.0+ / TOEFL 100+</t>
+        </is>
+      </c>
+      <c r="K152" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L152" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N152" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O152" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P152" s="64" t="inlineStr">
+        <is>
+          <t>Apply directly via UC Berkeley Mastercard Foundation Scholars page; highly competitive</t>
+        </is>
+      </c>
+      <c r="Q152" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R152" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="64" t="n">
+        <v>151</v>
+      </c>
+      <c r="B153" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- McGill University</t>
+        </is>
+      </c>
+      <c r="C153" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at McGill University</t>
+        </is>
+      </c>
+      <c r="D153" s="64" t="inlineStr">
+        <is>
+          <t>McGill University</t>
+        </is>
+      </c>
+      <c r="E153" s="64" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F153" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G153" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H153" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel + mentoring</t>
+        </is>
+      </c>
+      <c r="I153" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J153" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+</t>
+        </is>
+      </c>
+      <c r="K153" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L153" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M153" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N153" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O153" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P153" s="64" t="inlineStr">
+        <is>
+          <t>Apply directly via McGill Mastercard Foundation Scholars page</t>
+        </is>
+      </c>
+      <c r="Q153" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R153" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="64" t="n">
+        <v>152</v>
+      </c>
+      <c r="B154" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- Makerere University</t>
+        </is>
+      </c>
+      <c r="C154" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field) at Makerere University</t>
+        </is>
+      </c>
+      <c r="D154" s="64" t="inlineStr">
+        <is>
+          <t>Makerere University</t>
+        </is>
+      </c>
+      <c r="E154" s="64" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="F154" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G154" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H154" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + accommodation + mentoring</t>
+        </is>
+      </c>
+      <c r="I154" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J154" s="64" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K154" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L154" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M154" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N154" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O154" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P154" s="64" t="inlineStr">
+        <is>
+          <t>East African regional option -- easier logistics/lower cost of living than Western partners; apply directly via Makerere Mastercard Foundation office</t>
+        </is>
+      </c>
+      <c r="Q154" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R154" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="64" t="n">
+        <v>153</v>
+      </c>
+      <c r="B155" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- AIMS (African Institute for Mathematical Sciences)</t>
+        </is>
+      </c>
+      <c r="C155" s="64" t="inlineStr">
+        <is>
+          <t>MSc Mathematical Sciences</t>
+        </is>
+      </c>
+      <c r="D155" s="64" t="inlineStr">
+        <is>
+          <t>AIMS centres (Rwanda, Ghana, Senegal, South Africa, Tanzania, Cameroon)</t>
+        </is>
+      </c>
+      <c r="E155" s="64" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="F155" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G155" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H155" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + accommodation + stipend + travel within Africa</t>
+        </is>
+      </c>
+      <c r="I155" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J155" s="64" t="inlineStr">
+        <is>
+          <t>English or French</t>
+        </is>
+      </c>
+      <c r="K155" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L155" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M155" s="64" t="inlineStr">
+        <is>
+          <t>Medium-High</t>
+        </is>
+      </c>
+      <c r="N155" s="64" t="inlineStr">
+        <is>
+          <t>Mathematical Sciences / Data Science / Machine Learning</t>
+        </is>
+      </c>
+      <c r="O155" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P155" s="64" t="inlineStr">
+        <is>
+          <t>Relevant to Roy's energy data analysis background; intensive 1-year programme; strong alumni network in African tech and energy sectors</t>
+        </is>
+      </c>
+      <c r="Q155" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R155" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="64" t="n">
+        <v>154</v>
+      </c>
+      <c r="B156" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- University of Pretoria</t>
+        </is>
+      </c>
+      <c r="C156" s="64" t="inlineStr">
+        <is>
+          <t>Masters (any eligible field, strong engineering faculty) at University of Pretoria</t>
+        </is>
+      </c>
+      <c r="D156" s="64" t="inlineStr">
+        <is>
+          <t>University of Pretoria</t>
+        </is>
+      </c>
+      <c r="E156" s="64" t="inlineStr">
+        <is>
+          <t>South Africa</t>
+        </is>
+      </c>
+      <c r="F156" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G156" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H156" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + accommodation + mentoring</t>
+        </is>
+      </c>
+      <c r="I156" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J156" s="64" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K156" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L156" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M156" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N156" s="64" t="inlineStr">
+        <is>
+          <t>All fields including Engineering</t>
+        </is>
+      </c>
+      <c r="O156" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P156" s="64" t="inlineStr">
+        <is>
+          <t>Strong engineering and energy programmes; regional African option; apply via UP Mastercard Foundation office</t>
+        </is>
+      </c>
+      <c r="Q156" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R156" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="64" t="n">
+        <v>155</v>
+      </c>
+      <c r="B157" s="64" t="inlineStr">
+        <is>
+          <t>Mastercard Foundation Scholars -- African Leadership University (ALU)</t>
+        </is>
+      </c>
+      <c r="C157" s="64" t="inlineStr">
+        <is>
+          <t>Bachelor's and select Masters programmes, entrepreneurial leadership focus</t>
+        </is>
+      </c>
+      <c r="D157" s="64" t="inlineStr">
+        <is>
+          <t>ALU Rwanda</t>
+        </is>
+      </c>
+      <c r="E157" s="64" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="F157" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G157" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H157" s="64" t="inlineStr">
+        <is>
+          <t>Full and partial scholarships available</t>
+        </is>
+      </c>
+      <c r="I157" s="64" t="inlineStr">
+        <is>
+          <t>Varies</t>
+        </is>
+      </c>
+      <c r="J157" s="64" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K157" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L157" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M157" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N157" s="64" t="inlineStr">
+        <is>
+          <t>Entrepreneurship / Leadership / Business</t>
+        </is>
+      </c>
+      <c r="O157" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P157" s="64" t="inlineStr">
+        <is>
+          <t>Pan-African campus; practical leadership model; check current Masters offerings availability</t>
+        </is>
+      </c>
+      <c r="Q157" s="64" t="inlineStr">
+        <is>
+          <t>https://www.mastercardfdn.org/en/what-we-do/our-programs/mastercard-foundation-scholars-program/where-to-apply/</t>
+        </is>
+      </c>
+      <c r="R157" s="65" t="inlineStr">
+        <is>
+          <t>Global - Business</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="64" t="n">
+        <v>156</v>
+      </c>
+      <c r="B158" s="64" t="inlineStr">
+        <is>
+          <t>Clarendon Fund Scholarship</t>
+        </is>
+      </c>
+      <c r="C158" s="64" t="inlineStr">
+        <is>
+          <t>Masters or PhD, any subject at University of Oxford</t>
+        </is>
+      </c>
+      <c r="D158" s="64" t="inlineStr">
+        <is>
+          <t>University of Oxford</t>
+        </is>
+      </c>
+      <c r="E158" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F158" s="64" t="inlineStr">
+        <is>
+          <t>Dec 2026 - Jan 2027 (course-dependent)</t>
+        </is>
+      </c>
+      <c r="G158" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H158" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + college fees + living stipend</t>
+        </is>
+      </c>
+      <c r="I158" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J158" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 7.0+/TOEFL 100+ (Oxford standard)</t>
+        </is>
+      </c>
+      <c r="K158" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L158" s="64" t="n">
+        <v>76</v>
+      </c>
+      <c r="M158" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N158" s="64" t="inlineStr">
+        <is>
+          <t>All fields (Engineering Science, Energy Systems relevant)</t>
+        </is>
+      </c>
+      <c r="O158" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P158" s="64" t="inlineStr">
+        <is>
+          <t>Oxford's flagship scholarship, all nationalities, all subjects; automatically considered upon applying to an eligible Oxford graduate course; deadline typically follows Oxford's Jan graduate admissions round | LIVE-VERIFIED 2026-08-24: CONFIRMED: no separate application -- automatically considered when applying to an eligible Oxford graduate course by its Dec/Jan funding deadline. Check specific course page for exact date.</t>
+        </is>
+      </c>
+      <c r="Q158" s="64" t="inlineStr">
+        <is>
+          <t>https://www.ox.ac.uk/clarendon</t>
+        </is>
+      </c>
+      <c r="R158" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="64" t="n">
+        <v>157</v>
+      </c>
+      <c r="B159" s="64" t="inlineStr">
+        <is>
+          <t>Knight-Hennessy Scholars</t>
+        </is>
+      </c>
+      <c r="C159" s="64" t="inlineStr">
+        <is>
+          <t>Any graduate degree (Masters or PhD) at Stanford University</t>
+        </is>
+      </c>
+      <c r="D159" s="64" t="inlineStr">
+        <is>
+          <t>Stanford University</t>
+        </is>
+      </c>
+      <c r="E159" s="64" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F159" s="64" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G159" s="64" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="H159" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + living stipend + travel for full duration of degree</t>
+        </is>
+      </c>
+      <c r="I159" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J159" s="64" t="inlineStr">
+        <is>
+          <t>TOEFL 100+/IELTS 7.0+ (Stanford standard)</t>
+        </is>
+      </c>
+      <c r="K159" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L159" s="64" t="n">
+        <v>72</v>
+      </c>
+      <c r="M159" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N159" s="64" t="inlineStr">
+        <is>
+          <t>All fields (energy, engineering, public policy relevant)</t>
+        </is>
+      </c>
+      <c r="O159" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P159" s="64" t="inlineStr">
+        <is>
+          <t>Fully funded for entire Stanford graduate programme (up to 3 years); global leadership focus; extremely competitive but explicitly welcomes African applicants | LIVE-VERIFIED 2026-08-24: CONFIRMED: KHS application closes 6 Oct 2026, 1pm Pacific Time. Must also submit separate Stanford graduate degree application by the earlier of the KHS deadline or 1 Dec 2026.</t>
+        </is>
+      </c>
+      <c r="Q159" s="64" t="inlineStr">
+        <is>
+          <t>https://knight-hennessy.stanford.edu</t>
+        </is>
+      </c>
+      <c r="R159" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="64" t="n">
+        <v>158</v>
+      </c>
+      <c r="B160" s="64" t="inlineStr">
+        <is>
+          <t>Cambridge Trust Scholarship</t>
+        </is>
+      </c>
+      <c r="C160" s="64" t="inlineStr">
+        <is>
+          <t>Masters or PhD, any subject at University of Cambridge</t>
+        </is>
+      </c>
+      <c r="D160" s="64" t="inlineStr">
+        <is>
+          <t>University of Cambridge</t>
+        </is>
+      </c>
+      <c r="E160" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F160" s="64" t="inlineStr">
+        <is>
+          <t>Dec 2026 - Jan 2027 (course-dependent)</t>
+        </is>
+      </c>
+      <c r="G160" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H160" s="64" t="inlineStr">
+        <is>
+          <t>Full or partial: tuition + maintenance (varies by award type)</t>
+        </is>
+      </c>
+      <c r="I160" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J160" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 7.5+ (Cambridge standard)</t>
+        </is>
+      </c>
+      <c r="K160" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L160" s="64" t="n">
+        <v>70</v>
+      </c>
+      <c r="M160" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N160" s="64" t="inlineStr">
+        <is>
+          <t>All fields including Engineering for Sustainable Development</t>
+        </is>
+      </c>
+      <c r="O160" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P160" s="64" t="inlineStr">
+        <is>
+          <t>Broader than Gates Cambridge -- includes Cambridge Africa Scholarships and other Trust-funded awards; apply through Cambridge graduate admissions, funding considered automatically | LIVE-VERIFIED 2026-08-24: CONFIRMED: applications for 2027/28 entry open September 2026. Apply through course application in Applicant Portal by course-specific funding deadline (early Dec or early Jan).</t>
+        </is>
+      </c>
+      <c r="Q160" s="64" t="inlineStr">
+        <is>
+          <t>https://www.cambridgetrust.org</t>
+        </is>
+      </c>
+      <c r="R160" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="64" t="n">
+        <v>159</v>
+      </c>
+      <c r="B161" s="64" t="inlineStr">
+        <is>
+          <t>Commonwealth PhD Scholarship (Split-Site)</t>
+        </is>
+      </c>
+      <c r="C161" s="64" t="inlineStr">
+        <is>
+          <t>PhD, spend time at both home country and UK university, all fields</t>
+        </is>
+      </c>
+      <c r="D161" s="64" t="inlineStr">
+        <is>
+          <t>Various UK universities</t>
+        </is>
+      </c>
+      <c r="E161" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F161" s="64" t="inlineStr">
+        <is>
+          <t>SUSPENDED</t>
+        </is>
+      </c>
+      <c r="G161" s="64" t="inlineStr">
+        <is>
+          <t>SUSPENDED</t>
+        </is>
+      </c>
+      <c r="H161" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + flights for UK portion of study</t>
+        </is>
+      </c>
+      <c r="I161" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J161" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+</t>
+        </is>
+      </c>
+      <c r="K161" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L161" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M161" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N161" s="64" t="inlineStr">
+        <is>
+          <t>All fields (development-relevant preferred)</t>
+        </is>
+      </c>
+      <c r="O161" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P161" s="64" t="inlineStr">
+        <is>
+          <t>For PhD candidates already registered at a Kenyan university; funds a period of research at a UK university; Kenya on eligible country list | LIVE-VERIFIED 2026-08-24: CONFIRMED: programme is currently under review and NOT running for the 2026/27 cycle. No 2027 deadline exists. Check cscuk.fcdo.gov.uk periodically for programme reinstatement.</t>
+        </is>
+      </c>
+      <c r="Q161" s="64" t="inlineStr">
+        <is>
+          <t>https://cscuk.fcdo.gov.uk</t>
+        </is>
+      </c>
+      <c r="R161" s="65" t="inlineStr">
+        <is>
+          <t>Global - Public Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="64" t="n">
+        <v>160</v>
+      </c>
+      <c r="B162" s="64" t="inlineStr">
+        <is>
+          <t>Commonwealth Rutherford Fellowship</t>
+        </is>
+      </c>
+      <c r="C162" s="64" t="inlineStr">
+        <is>
+          <t>Postdoctoral research fellowship (1-3 years) at UK universities</t>
+        </is>
+      </c>
+      <c r="D162" s="64" t="inlineStr">
+        <is>
+          <t>Various UK universities</t>
+        </is>
+      </c>
+      <c r="E162" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F162" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G162" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H162" s="64" t="inlineStr">
+        <is>
+          <t>Full: salary + research costs + travel</t>
+        </is>
+      </c>
+      <c r="I162" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J162" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+</t>
+        </is>
+      </c>
+      <c r="K162" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="L162" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M162" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N162" s="64" t="inlineStr">
+        <is>
+          <t>All fields (research focus)</t>
+        </is>
+      </c>
+      <c r="O162" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P162" s="64" t="inlineStr">
+        <is>
+          <t>For early-career researchers who already hold a PhD; not a taught masters; Kenya eligible as Commonwealth member | LIVE-VERIFIED 2026-08-24: No 2027 deadline published yet in search results -- monitor cscuk.fcdo.gov.uk directly.</t>
+        </is>
+      </c>
+      <c r="Q162" s="64" t="inlineStr">
+        <is>
+          <t>https://cscuk.fcdo.gov.uk</t>
+        </is>
+      </c>
+      <c r="R162" s="65" t="inlineStr">
+        <is>
+          <t>Global - Sciences</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="64" t="n">
+        <v>161</v>
+      </c>
+      <c r="B163" s="64" t="inlineStr">
+        <is>
+          <t>Yenching Academy Scholarship</t>
+        </is>
+      </c>
+      <c r="C163" s="64" t="inlineStr">
+        <is>
+          <t>One-year interdisciplinary Master's in China Studies</t>
+        </is>
+      </c>
+      <c r="D163" s="64" t="inlineStr">
+        <is>
+          <t>Peking University</t>
+        </is>
+      </c>
+      <c r="E163" s="64" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F163" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G163" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H163" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + accommodation + stipend + travel + research/language trips</t>
+        </is>
+      </c>
+      <c r="I163" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J163" s="64" t="inlineStr">
+        <is>
+          <t>English (China Studies taught in English)</t>
+        </is>
+      </c>
+      <c r="K163" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L163" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M163" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N163" s="64" t="inlineStr">
+        <is>
+          <t>Area Studies / Economics / Public Policy / Politics (China-Africa relations track available)</t>
+        </is>
+      </c>
+      <c r="O163" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P163" s="64" t="inlineStr">
+        <is>
+          <t>Fully funded, global cohort model with strong African representation historically; relevant for those interested in China-Africa energy and development ties | LIVE-VERIFIED 2026-08-24: CONFIRMED: 2027 cohort recruitment information will be released around September 2026. Typical direct-applicant deadline falls Dec-Jan. Monitor yenchingacademy.pku.edu.cn from September.</t>
+        </is>
+      </c>
+      <c r="Q163" s="64" t="inlineStr">
+        <is>
+          <t>https://yenchingacademy.pku.edu.cn</t>
+        </is>
+      </c>
+      <c r="R163" s="65" t="inlineStr">
+        <is>
+          <t>Global - Social Sciences</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="64" t="n">
+        <v>162</v>
+      </c>
+      <c r="B164" s="64" t="inlineStr">
+        <is>
+          <t>Schwarzman Scholars</t>
+        </is>
+      </c>
+      <c r="C164" s="64" t="inlineStr">
+        <is>
+          <t>One-year Master's in Global Affairs</t>
+        </is>
+      </c>
+      <c r="D164" s="64" t="inlineStr">
+        <is>
+          <t>Tsinghua University</t>
+        </is>
+      </c>
+      <c r="E164" s="64" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="F164" s="64" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="G164" s="64" t="inlineStr">
+        <is>
+          <t>URGENT - 16 DAYS REMAINING</t>
+        </is>
+      </c>
+      <c r="H164" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + room/board + travel + stipend + laptop</t>
+        </is>
+      </c>
+      <c r="I164" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J164" s="64" t="inlineStr">
+        <is>
+          <t>English (Global Affairs taught in English)</t>
+        </is>
+      </c>
+      <c r="K164" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L164" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M164" s="64" t="inlineStr">
+        <is>
+          <t>Extremely High</t>
+        </is>
+      </c>
+      <c r="N164" s="64" t="inlineStr">
+        <is>
+          <t>Public Policy / Global Affairs / Economics / Business</t>
+        </is>
+      </c>
+      <c r="O164" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P164" s="64" t="inlineStr">
+        <is>
+          <t>Highly selective global leadership programme; explicitly recruits from Africa; strong alumni network | LIVE-VERIFIED 2026-08-24: CONFIRMED: US/Global application deadline is 9 September 2026, 3pm EDT. Application opened 8 April 2026. Separate earlier deadline exists for China-region applicants (20 May 2026) -- not applicable to Kenya.</t>
+        </is>
+      </c>
+      <c r="Q164" s="64" t="inlineStr">
+        <is>
+          <t>https://www.schwarzmanscholars.org</t>
+        </is>
+      </c>
+      <c r="R164" s="65" t="inlineStr">
+        <is>
+          <t>Global - Public Policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="64" t="n">
+        <v>163</v>
+      </c>
+      <c r="B165" s="64" t="inlineStr">
+        <is>
+          <t>Weidenfeld-Hoffmann Scholarship and Leadership Programme</t>
+        </is>
+      </c>
+      <c r="C165" s="64" t="inlineStr">
+        <is>
+          <t>Masters at University of Oxford in fields relevant to good governance and economic development</t>
+        </is>
+      </c>
+      <c r="D165" s="64" t="inlineStr">
+        <is>
+          <t>University of Oxford</t>
+        </is>
+      </c>
+      <c r="E165" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F165" s="64" t="inlineStr">
+        <is>
+          <t>2027-01-08</t>
+        </is>
+      </c>
+      <c r="G165" s="64" t="inlineStr">
+        <is>
+          <t>OPEN NOW - 342 DAYS REMAINING</t>
+        </is>
+      </c>
+      <c r="H165" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + college fees + living stipend + leadership training</t>
+        </is>
+      </c>
+      <c r="I165" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J165" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 7.0+ (Oxford standard)</t>
+        </is>
+      </c>
+      <c r="K165" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L165" s="64" t="n">
+        <v>68</v>
+      </c>
+      <c r="M165" s="64" t="inlineStr">
+        <is>
+          <t>Very High</t>
+        </is>
+      </c>
+      <c r="N165" s="64" t="inlineStr">
+        <is>
+          <t>Public Policy / Economics / Development / Energy Policy</t>
+        </is>
+      </c>
+      <c r="O165" s="64" t="inlineStr">
+        <is>
+          <t>LE</t>
+        </is>
+      </c>
+      <c r="P165" s="64" t="inlineStr">
+        <is>
+          <t>For students from developing/transition countries; leadership development component alongside degree; Kenya eligible | LIVE-VERIFIED 2026-08-24: CONFIRMED: deadline 8 January 2027 (varies slightly by specific graduate course, generally Dec 2026-Jan 2027). Interviews for shortlisted candidates held late April/early May 2027.</t>
+        </is>
+      </c>
+      <c r="Q165" s="64" t="inlineStr">
+        <is>
+          <t>https://www.weidenfeldhoffmann.com</t>
+        </is>
+      </c>
+      <c r="R165" s="78" t="inlineStr">
+        <is>
+          <t>Roy Priority</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="64" t="n">
+        <v>164</v>
+      </c>
+      <c r="B166" s="64" t="inlineStr">
+        <is>
+          <t>AAUW International Fellowship</t>
+        </is>
+      </c>
+      <c r="C166" s="64" t="inlineStr">
+        <is>
+          <t>Masters or PhD at accredited US universities (women only)</t>
+        </is>
+      </c>
+      <c r="D166" s="64" t="inlineStr">
+        <is>
+          <t>Various US universities</t>
+        </is>
+      </c>
+      <c r="E166" s="64" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F166" s="64" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="G166" s="64" t="inlineStr">
+        <is>
+          <t>URGENT - 24 DAYS REMAINING</t>
+        </is>
+      </c>
+      <c r="H166" s="64" t="inlineStr">
+        <is>
+          <t>Full or partial: tuition + stipend (varies by fellowship type)</t>
+        </is>
+      </c>
+      <c r="I166" s="64" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J166" s="64" t="inlineStr">
+        <is>
+          <t>TOEFL/IELTS (institution standard)</t>
+        </is>
+      </c>
+      <c r="K166" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L166" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M166" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N166" s="64" t="inlineStr">
+        <is>
+          <t>All fields</t>
+        </is>
+      </c>
+      <c r="O166" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P166" s="64" t="inlineStr">
+        <is>
+          <t>Restricted to women applicants; Kenya eligible; long-running American Association of University Women programme | LIVE-VERIFIED 2026-08-24: CONFIRMED: applications opened 17 Aug 2026, deadline 17 Sept 2026, 5pm ET. Programme must start on or before 15 Sept 2027.</t>
+        </is>
+      </c>
+      <c r="Q166" s="64" t="inlineStr">
+        <is>
+          <t>https://www.aauw.org/resources/programs/fellowships-grants/</t>
+        </is>
+      </c>
+      <c r="R166" s="65" t="inlineStr">
+        <is>
+          <t>Global - Education</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="64" t="n">
+        <v>165</v>
+      </c>
+      <c r="B167" s="64" t="inlineStr">
+        <is>
+          <t>Zonta International Amelia Earhart Fellowship</t>
+        </is>
+      </c>
+      <c r="C167" s="64" t="inlineStr">
+        <is>
+          <t>PhD in aerospace-related sciences and engineering (women only)</t>
+        </is>
+      </c>
+      <c r="D167" s="64" t="inlineStr">
+        <is>
+          <t>Various universities worldwide</t>
+        </is>
+      </c>
+      <c r="E167" s="64" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="F167" s="64" t="inlineStr">
+        <is>
+          <t>2026-11-15</t>
+        </is>
+      </c>
+      <c r="G167" s="64" t="inlineStr">
+        <is>
+          <t>OPEN NOW - 83 DAYS REMAINING</t>
+        </is>
+      </c>
+      <c r="H167" s="64" t="inlineStr">
+        <is>
+          <t>Award: USD 10,000 (partial support)</t>
+        </is>
+      </c>
+      <c r="I167" s="64" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J167" s="64" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K167" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L167" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M167" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N167" s="64" t="inlineStr">
+        <is>
+          <t>Aerospace Engineering / Space Sciences (women only)</t>
+        </is>
+      </c>
+      <c r="O167" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P167" s="64" t="inlineStr">
+        <is>
+          <t>Restricted to women pursuing PhD; niche field (aerospace); Kenya eligible as open international competition | LIVE-VERIFIED 2026-08-24: CONFIRMED: deadline for current fellowship cycle is 15 November 2026. Check zonta.org/AEFellowship for exact application portal opening.</t>
+        </is>
+      </c>
+      <c r="Q167" s="64" t="inlineStr">
+        <is>
+          <t>https://www.zonta.org/Web/Programs/Amelia_Earhart_Fellowship/</t>
+        </is>
+      </c>
+      <c r="R167" s="65" t="inlineStr">
+        <is>
+          <t>Global - Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="64" t="n">
+        <v>166</v>
+      </c>
+      <c r="B168" s="64" t="inlineStr">
+        <is>
+          <t>Schlumberger Foundation Faculty for the Future</t>
+        </is>
+      </c>
+      <c r="C168" s="64" t="inlineStr">
+        <is>
+          <t>PhD in STEM fields at top international universities (women only, from developing countries)</t>
+        </is>
+      </c>
+      <c r="D168" s="64" t="inlineStr">
+        <is>
+          <t>Selected top-ranked universities worldwide</t>
+        </is>
+      </c>
+      <c r="E168" s="64" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="F168" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G168" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H168" s="64" t="inlineStr">
+        <is>
+          <t>Full: tuition + stipend + travel</t>
+        </is>
+      </c>
+      <c r="I168" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J168" s="64" t="inlineStr">
+        <is>
+          <t>English (institution standard)</t>
+        </is>
+      </c>
+      <c r="K168" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L168" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M168" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N168" s="64" t="inlineStr">
+        <is>
+          <t>STEM -- Physical Sciences, Engineering, Mathematics, Computer Science</t>
+        </is>
+      </c>
+      <c r="O168" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P168" s="64" t="inlineStr">
+        <is>
+          <t>Restricted to women in STEM PhD programmes intending to return to teach in home country; Kenya explicitly eligible; highly relevant for African women engineers | LIVE-VERIFIED 2026-08-24: Most recent confirmed deadline (2026-2027 cycle) was 7 Nov 2025, already closed. Next cycle (2027-2028) not yet announced -- historically opens around Aug-Sep with deadline Oct-Nov. Monitor fftf.slb.com.</t>
+        </is>
+      </c>
+      <c r="Q168" s="64" t="inlineStr">
+        <is>
+          <t>https://facultyforthefuture.net</t>
+        </is>
+      </c>
+      <c r="R168" s="65" t="inlineStr">
+        <is>
+          <t>Global - Sciences</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="64" t="n">
+        <v>167</v>
+      </c>
+      <c r="B169" s="64" t="inlineStr">
+        <is>
+          <t>GREAT Scholarships (British Council)</t>
+        </is>
+      </c>
+      <c r="C169" s="64" t="inlineStr">
+        <is>
+          <t>Masters at partner UK universities (country-specific allocation)</t>
+        </is>
+      </c>
+      <c r="D169" s="64" t="inlineStr">
+        <is>
+          <t>Various UK universities (partner list varies by year)</t>
+        </is>
+      </c>
+      <c r="E169" s="64" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="F169" s="64" t="inlineStr">
+        <is>
+          <t>Check website (varies by partner university)</t>
+        </is>
+      </c>
+      <c r="G169" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H169" s="64" t="inlineStr">
+        <is>
+          <t>Full or partial: GBP 10,000+ tuition contribution (varies by university)</t>
+        </is>
+      </c>
+      <c r="I169" s="64" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="J169" s="64" t="inlineStr">
+        <is>
+          <t>IELTS 6.5+</t>
+        </is>
+      </c>
+      <c r="K169" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L169" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M169" s="64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N169" s="64" t="inlineStr">
+        <is>
+          <t>Varies by partner university and year</t>
+        </is>
+      </c>
+      <c r="O169" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P169" s="64" t="inlineStr">
+        <is>
+          <t>British Council programme; country allocation changes annually -- verify whether Kenya is on the current year's eligible country list before applying | LIVE-VERIFIED 2026-08-24: CONFIRMED: Kenya IS on the eligible country list for the 2026-27 cycle (confirmed via study-uk.britishcouncil.org/scholarships-funding/great-scholarships/kenya). GBP 10,000+ towards one-year taught postgraduate tuition at 60 partner UK universities. Deadlines set individually by each partner university, typically Jan-Jun for Sept entry.</t>
+        </is>
+      </c>
+      <c r="Q169" s="64" t="inlineStr">
+        <is>
+          <t>https://study-uk.britishcouncil.org/scholarships/great-scholarships</t>
+        </is>
+      </c>
+      <c r="R169" s="65" t="inlineStr">
+        <is>
+          <t>Global - Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="64" t="n">
+        <v>168</v>
+      </c>
+      <c r="B170" s="64" t="inlineStr">
+        <is>
+          <t>L'Oreal-UNESCO For Women in Science Fellowship</t>
+        </is>
+      </c>
+      <c r="C170" s="64" t="inlineStr">
+        <is>
+          <t>PhD or postdoctoral fellowship in life/physical sciences (women only)</t>
+        </is>
+      </c>
+      <c r="D170" s="64" t="inlineStr">
+        <is>
+          <t>Home institution or international host</t>
+        </is>
+      </c>
+      <c r="E170" s="64" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="F170" s="64" t="inlineStr">
+        <is>
+          <t>Check website</t>
+        </is>
+      </c>
+      <c r="G170" s="64" t="inlineStr">
+        <is>
+          <t>CHECK WEBSITE</t>
+        </is>
+      </c>
+      <c r="H170" s="64" t="inlineStr">
+        <is>
+          <t>Fellowship award (varies by region -- Sub-Saharan Africa programme exists)</t>
+        </is>
+      </c>
+      <c r="I170" s="64" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J170" s="64" t="inlineStr">
+        <is>
+          <t>English or French</t>
+        </is>
+      </c>
+      <c r="K170" s="64" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="L170" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="M170" s="64" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N170" s="64" t="inlineStr">
+        <is>
+          <t>Life Sciences / Physical Sciences / Engineering (women only)</t>
+        </is>
+      </c>
+      <c r="O170" s="64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P170" s="64" t="inlineStr">
+        <is>
+          <t>Sub-Saharan Africa regional programme exists specifically; Kenya eligible; supports women researchers at PhD and postdoc level | LIVE-VERIFIED 2026-08-24: Most recent confirmed Sub-Saharan Africa deadline was 17 April 2026, already closed. Next cycle deadline not yet announced -- historically opens Feb-Mar. Monitor forwomeninscience.com/authority/sub-saharan-africa---regional-program.</t>
+        </is>
+      </c>
+      <c r="Q170" s="64" t="inlineStr">
+        <is>
+          <t>https://www.forwomeninscience.com</t>
+        </is>
+      </c>
+      <c r="R170" s="65" t="inlineStr">
         <is>
           <t>Global - Sciences</t>
         </is>

</xml_diff>